<commit_message>
Data and figures updated
</commit_message>
<xml_diff>
--- a/src/New-release/Figure6.xlsx
+++ b/src/New-release/Figure6.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\visualisations\dvc3400-3499\dvc3420-productivity-flash\fig6\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ostsue\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7693464E-6CD1-416F-8948-A1317D30C8C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E799793D-D2FC-41AF-AC51-FF2AD342B410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="672" yWindow="696" windowWidth="19116" windowHeight="10092" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="datadownload" sheetId="1" r:id="rId1"/>
+    <sheet name="Data for Dataviz" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -52,7 +52,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
       </rPr>
       <t xml:space="preserve">1. </t>
     </r>
@@ -61,7 +60,6 @@
         <sz val="10"/>
         <color rgb="FF323132"/>
         <rFont val="Arial"/>
-        <family val="2"/>
       </rPr>
       <t>The industry contributions may not add up to the total growth in output per hour. This is due to the National Accounts balancing value and the impact of rounding.</t>
     </r>
@@ -155,7 +153,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -172,13 +170,11 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF323132"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -540,24 +536,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="60.33203125" customWidth="1"/>
-    <col min="2" max="2" width="20.5546875" customWidth="1"/>
-    <col min="3" max="3" width="17.6640625" customWidth="1"/>
+    <col min="1" max="1" width="38.28515625" customWidth="1"/>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -566,28 +562,28 @@
       </c>
       <c r="C4" s="1"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3">
       <c r="B5" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="1"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3">
       <c r="B6" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="1"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3">
       <c r="C7" s="1"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3">
       <c r="C8" s="1"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3">
       <c r="C9" s="1"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -595,7 +591,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -606,7 +602,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" ht="15">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -617,222 +613,223 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" ht="15">
       <c r="A14" t="s">
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <v>2.5325785191873399E-2</v>
+        <v>2.5372118454875001E-2</v>
       </c>
       <c r="C14" s="2">
         <v>6.9091985072051998E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" ht="15">
       <c r="A15" t="s">
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>1.4039633533439799E-2</v>
+        <v>1.4008211608446799E-2</v>
       </c>
       <c r="C15" s="2">
         <v>8.6069359491453903E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" ht="15">
       <c r="A16" t="s">
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <v>1.0459754026746999E-2</v>
+        <v>1.0507311390668199E-2</v>
       </c>
       <c r="C16" s="2">
         <v>0.11046921711254699</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="15">
       <c r="A17" t="s">
         <v>15</v>
       </c>
       <c r="B17" s="2">
-        <v>7.16752854171582E-3</v>
+        <v>6.8662467350352092E-3</v>
       </c>
       <c r="C17" s="2">
         <v>6.8666704517909793E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" ht="15">
       <c r="A18" t="s">
         <v>16</v>
       </c>
       <c r="B18" s="2">
-        <v>6.4390464326143804E-3</v>
+        <v>6.4282357939118998E-3</v>
       </c>
       <c r="C18" s="2">
         <v>5.6393074969482399E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" ht="15">
       <c r="A19" t="s">
         <v>17</v>
       </c>
       <c r="B19" s="2">
-        <v>3.7715005086695901E-3</v>
+        <v>3.7802879275062899E-3</v>
       </c>
       <c r="C19" s="2">
         <v>4.4110710518787601E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" ht="15">
       <c r="A20" t="s">
         <v>18</v>
       </c>
       <c r="B20" s="2">
-        <v>1.5156808385038999E-3</v>
+        <v>1.5291339024912302E-3</v>
       </c>
       <c r="C20" s="2">
         <v>7.0960162294484101E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" ht="15">
       <c r="A21" t="s">
         <v>19</v>
       </c>
       <c r="B21" s="2">
-        <v>3.4345937538899003E-4</v>
+        <v>3.4581462539639901E-4</v>
       </c>
       <c r="C21" s="2">
         <v>1.33884214502994E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" ht="15">
       <c r="A22" t="s">
         <v>20</v>
       </c>
       <c r="B22" s="2">
-        <v>1.3398950016232499E-4</v>
+        <v>1.8606209632966901E-4</v>
       </c>
       <c r="C22" s="2">
         <v>5.3101108677470199E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" ht="15">
       <c r="A23" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="2">
-        <v>-2.7394617580237001E-4</v>
+        <v>-2.0695079802495099E-4</v>
       </c>
       <c r="C23" s="2">
         <v>6.3176272511480905E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" ht="15">
       <c r="A24" t="s">
         <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>-1.4504694979601501E-3</v>
+        <v>-1.4205561423764198E-3</v>
       </c>
       <c r="C24" s="2">
         <v>1.64363564102172E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" ht="15">
       <c r="A25" t="s">
         <v>23</v>
       </c>
       <c r="B25" s="2">
-        <v>-1.53039371054455E-3</v>
+        <v>-1.5405008116719399E-3</v>
       </c>
       <c r="C25" s="2">
         <v>2.11908729006208E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" ht="15">
       <c r="A26" t="s">
         <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>-2.0866418793098599E-3</v>
+        <v>-2.0872171286142401E-3</v>
       </c>
       <c r="C26" s="2">
         <v>1.11561079895967E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" ht="15">
       <c r="A27" t="s">
         <v>25</v>
       </c>
       <c r="B27" s="2">
-        <v>-2.8175579083962298E-3</v>
+        <v>-2.79491094728153E-3</v>
       </c>
       <c r="C27" s="2">
         <v>3.2992817726610599E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" ht="15">
       <c r="A28" t="s">
         <v>26</v>
       </c>
       <c r="B28" s="2">
-        <v>-3.1014163639112801E-3</v>
+        <v>-3.06179373114731E-3</v>
       </c>
       <c r="C28" s="2">
         <v>0.113281309711245</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" ht="15">
       <c r="A29" t="s">
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>-5.4457099979588197E-3</v>
+        <v>-5.4368020070388601E-3</v>
       </c>
       <c r="C29" s="2">
         <v>4.3964400905809303E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" ht="15">
       <c r="A30" t="s">
         <v>28</v>
       </c>
       <c r="B30" s="2">
-        <v>-8.5237933034656294E-3</v>
+        <v>-8.5224120230683806E-3</v>
       </c>
       <c r="C30" s="2">
         <v>1.6158477331836701E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" ht="15">
       <c r="A31" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="2">
-        <v>-9.2305032889186608E-3</v>
+        <v>-9.2487728274891195E-3</v>
       </c>
       <c r="C31" s="2">
         <v>8.3735502791893096E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" ht="15">
       <c r="A32" t="s">
         <v>30</v>
       </c>
       <c r="B32" s="2">
-        <v>-1.2188849385983301E-2</v>
+        <v>-1.2151286566558299E-2</v>
       </c>
       <c r="C32" s="2">
         <v>8.9521283681237199E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" ht="15">
       <c r="A33" t="s">
         <v>31</v>
       </c>
       <c r="B33" s="2">
-        <v>-3.4205582798278999E-5</v>
-      </c>
+        <v>-3.9328697323535097E-5</v>
+      </c>
+      <c r="C33" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -851,8 +848,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E0CEF6E26CBF2C4F8000DAAA032CD586" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="156efd3b4c34ab36c49a3cc1bad9b9a6">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8a54c791-04d1-4dd7-97a3-a882d4048403" xmlns:ns3="7c97fbf4-89e8-4607-8aa6-eba0d12e3a2a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1c801130155331743e24030937d8c3da" ns2:_="" ns3:_="">
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E0CEF6E26CBF2C4F8000DAAA032CD586" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3825d4c36eddbd19ff5877cf568b1130">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8a54c791-04d1-4dd7-97a3-a882d4048403" xmlns:ns3="7c97fbf4-89e8-4607-8aa6-eba0d12e3a2a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="20db92a579f18a3b40827b4b7272a8b7" ns2:_="" ns3:_="">
     <xsd:import namespace="8a54c791-04d1-4dd7-97a3-a882d4048403"/>
     <xsd:import namespace="7c97fbf4-89e8-4607-8aa6-eba0d12e3a2a"/>
     <xsd:element name="properties">
@@ -1099,49 +1105,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EDAD2DC3-87EC-4167-B2AD-C5DBB7ECB4E8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="8a54c791-04d1-4dd7-97a3-a882d4048403"/>
-    <ds:schemaRef ds:uri="7c97fbf4-89e8-4607-8aa6-eba0d12e3a2a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EDAD2DC3-87EC-4167-B2AD-C5DBB7ECB4E8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5127BBF4-6353-450E-9162-146089B209A6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="8a54c791-04d1-4dd7-97a3-a882d4048403"/>
-    <ds:schemaRef ds:uri="7c97fbf4-89e8-4607-8aa6-eba0d12e3a2a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8557CAEA-ABFE-4BAB-A82C-A482A20DAFD5}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8557CAEA-ABFE-4BAB-A82C-A482A20DAFD5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FD4B0C1-33E8-4E1F-95C6-2EBE429A960E}"/>
 </file>
</xml_diff>